<commit_message>
fixed api for payroll
</commit_message>
<xml_diff>
--- a/public/templates/cos/payslip.xlsx
+++ b/public/templates/cos/payslip.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DOST\OneDrive\Documents\COS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB9416D-57BA-44E7-8195-24780B435878}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCD1AE34-D6E2-4B9E-8433-93BDDCD37645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4D00BDC9-532D-4D12-A161-F58336A59D96}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="PAYSLIP" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">PAYSLIP!$A$1:$BA$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">PAYSLIP!$A$1:$M$18</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,13 +37,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t xml:space="preserve">      TECHNOLOGY APPLICATION AND PROMOTION INSTITUTE</t>
-  </si>
-  <si>
-    <t>***** PAY SLIP *****
-for the month of APRIL 2024</t>
   </si>
   <si>
     <t>NAME</t>
@@ -341,7 +337,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
@@ -360,61 +356,116 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -426,66 +477,21 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -951,7 +957,7 @@
   <sheetPr codeName="Sheet37">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.5546875" customWidth="1"/>
@@ -964,43 +970,45 @@
     <col min="9" max="9" width="9.109375" customWidth="1"/>
     <col min="10" max="10" width="7.109375" customWidth="1"/>
     <col min="11" max="11" width="2.33203125" customWidth="1"/>
-    <col min="12" max="12" width="14.44140625" customWidth="1"/>
-    <col min="13" max="13" width="4.88671875" customWidth="1"/>
-    <col min="14" max="16384" width="9.109375" hidden="1"/>
+    <col min="12" max="12" width="16.6640625" customWidth="1"/>
+    <col min="13" max="13" width="8.21875" customWidth="1"/>
+    <col min="14" max="15" width="9.109375" customWidth="1"/>
+    <col min="16" max="16" width="0" hidden="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.109375" hidden="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
-      <c r="I2" s="51"/>
-      <c r="J2" s="51"/>
-      <c r="K2" s="51"/>
-      <c r="L2" s="51"/>
-      <c r="M2" s="51"/>
+      <c r="B2" s="36"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
     </row>
     <row r="3" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="51"/>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51"/>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="51"/>
-      <c r="J3" s="51"/>
-      <c r="K3" s="51"/>
-      <c r="L3" s="51"/>
-      <c r="M3" s="51"/>
+      <c r="A3" s="36"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="36"/>
+      <c r="H3" s="36"/>
+      <c r="I3" s="36"/>
+      <c r="J3" s="36"/>
+      <c r="K3" s="36"/>
+      <c r="L3" s="36"/>
+      <c r="M3" s="36"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
@@ -1018,54 +1026,52 @@
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="1:13" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="52" t="s">
+      <c r="A5" s="37"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="38"/>
+      <c r="I5" s="38"/>
+      <c r="J5" s="38"/>
+      <c r="K5" s="38"/>
+      <c r="L5" s="38"/>
+      <c r="M5" s="39"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="53"/>
-      <c r="C5" s="53"/>
-      <c r="D5" s="53"/>
-      <c r="E5" s="53"/>
-      <c r="F5" s="53"/>
-      <c r="G5" s="53"/>
-      <c r="H5" s="53"/>
-      <c r="I5" s="53"/>
-      <c r="J5" s="53"/>
-      <c r="K5" s="53"/>
-      <c r="L5" s="53"/>
-      <c r="M5" s="54"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" s="55"/>
-      <c r="D6" s="55"/>
-      <c r="E6" s="55"/>
-      <c r="F6" s="55"/>
-      <c r="G6" s="55"/>
-      <c r="H6" s="55"/>
-      <c r="I6" s="56"/>
-      <c r="J6" s="56"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="40"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="40"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
       <c r="K6" s="4"/>
       <c r="L6" s="5"/>
       <c r="M6" s="6"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
-      <c r="C7" s="57"/>
-      <c r="D7" s="57"/>
-      <c r="E7" s="57"/>
-      <c r="F7" s="57"/>
-      <c r="G7" s="57"/>
-      <c r="H7" s="57"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="42"/>
+      <c r="H7" s="42"/>
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
       <c r="K7" s="9"/>
@@ -1073,185 +1079,185 @@
       <c r="M7" s="10"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A8" s="48" t="s">
+      <c r="A8" s="43" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="44"/>
+      <c r="C8" s="45"/>
+      <c r="D8" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="49"/>
-      <c r="C8" s="50"/>
-      <c r="D8" s="48" t="s">
+      <c r="E8" s="45"/>
+      <c r="F8" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="50"/>
-      <c r="F8" s="48" t="s">
+      <c r="G8" s="44"/>
+      <c r="H8" s="45"/>
+      <c r="I8" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="G8" s="49"/>
-      <c r="H8" s="50"/>
-      <c r="I8" s="48" t="s">
+      <c r="J8" s="44"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="J8" s="49"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="48" t="s">
+      <c r="M8" s="45"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A9" s="49"/>
+      <c r="B9" s="50"/>
+      <c r="C9" s="50"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="50"/>
+      <c r="G9" s="50"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="50"/>
+      <c r="J9" s="50"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="19"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A10" s="46"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="48"/>
+      <c r="J10" s="48"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="18"/>
+      <c r="M10" s="12"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A11" s="46"/>
+      <c r="B11" s="47"/>
+      <c r="C11" s="47"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="47"/>
+      <c r="G11" s="47"/>
+      <c r="H11" s="47"/>
+      <c r="I11" s="58"/>
+      <c r="J11" s="58"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="18"/>
+      <c r="M11" s="12"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A12" s="28"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="30"/>
+      <c r="K12" s="23"/>
+      <c r="L12" s="31"/>
+      <c r="M12" s="20"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A13" s="59"/>
+      <c r="B13" s="58"/>
+      <c r="C13" s="58"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="58"/>
+      <c r="G13" s="58"/>
+      <c r="H13" s="58"/>
+      <c r="I13" s="58"/>
+      <c r="J13" s="58"/>
+      <c r="K13" s="23"/>
+      <c r="L13" s="23"/>
+      <c r="M13" s="20"/>
+    </row>
+    <row r="14" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="32"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="27"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="33"/>
+      <c r="M14" s="20"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A15" s="54"/>
+      <c r="B15" s="55"/>
+      <c r="C15" s="55"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="56"/>
+      <c r="G15" s="56"/>
+      <c r="H15" s="56"/>
+      <c r="I15" s="35"/>
+      <c r="J15" s="35"/>
+      <c r="K15" s="35"/>
+      <c r="L15" s="35"/>
+      <c r="M15" s="21"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A16" s="57"/>
+      <c r="B16" s="57"/>
+      <c r="C16" s="57"/>
+      <c r="D16" s="57"/>
+      <c r="E16" s="57"/>
+      <c r="F16" s="57"/>
+      <c r="G16" s="57"/>
+      <c r="H16" s="57"/>
+      <c r="I16" s="57"/>
+      <c r="J16" s="57"/>
+      <c r="K16" s="57"/>
+      <c r="L16" s="57"/>
+      <c r="M16" s="57"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A17" s="14"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="M8" s="50"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A9" s="47"/>
-      <c r="B9" s="35"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="35"/>
-      <c r="I9" s="35"/>
-      <c r="J9" s="35"/>
-      <c r="K9" s="13"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="14"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A10" s="45"/>
-      <c r="B10" s="46"/>
-      <c r="C10" s="46"/>
-      <c r="D10" s="58"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="34"/>
-      <c r="I10" s="60"/>
-      <c r="J10" s="60"/>
-      <c r="K10" s="12"/>
-      <c r="L10" s="61"/>
-      <c r="M10" s="20"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" s="33"/>
-      <c r="B11" s="34"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="34"/>
-      <c r="H11" s="34"/>
-      <c r="I11" s="59"/>
-      <c r="J11" s="59"/>
-      <c r="K11" s="12"/>
-      <c r="L11" s="61"/>
-      <c r="M11" s="20"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="21"/>
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="12"/>
-      <c r="L12" s="26"/>
-      <c r="M12" s="17"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" s="36"/>
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="37"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="37"/>
-      <c r="I13" s="37"/>
-      <c r="J13" s="37"/>
-      <c r="K13" s="12"/>
-      <c r="L13" s="12"/>
-      <c r="M13" s="17"/>
-    </row>
-    <row r="14" spans="1:13" ht="16.2" x14ac:dyDescent="0.45">
-      <c r="A14" s="15"/>
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="H14" s="16"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="16"/>
-      <c r="K14" s="12"/>
-      <c r="L14" s="27"/>
-      <c r="M14" s="17"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" s="41"/>
-      <c r="B15" s="42"/>
-      <c r="C15" s="42"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="43"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="43"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9"/>
-      <c r="M15" s="10"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" s="44"/>
-      <c r="B16" s="44"/>
-      <c r="C16" s="44"/>
-      <c r="D16" s="44"/>
-      <c r="E16" s="44"/>
-      <c r="F16" s="44"/>
-      <c r="G16" s="44"/>
-      <c r="H16" s="44"/>
-      <c r="I16" s="44"/>
-      <c r="J16" s="44"/>
-      <c r="K16" s="44"/>
-      <c r="L16" s="44"/>
-      <c r="M16" s="44"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A17" s="29"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="38" t="s">
+      <c r="D17" s="51"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="52" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="38"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="39" t="s">
+      <c r="G17" s="52"/>
+      <c r="H17" s="52"/>
+      <c r="I17" s="52"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="14"/>
+      <c r="L17" s="14"/>
+      <c r="M17" s="14"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A18" s="17"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="G17" s="39"/>
-      <c r="H17" s="39"/>
-      <c r="I17" s="39"/>
-      <c r="J17" s="31"/>
-      <c r="K17" s="29"/>
-      <c r="L17" s="29"/>
-      <c r="M17" s="29"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A18" s="32"/>
-      <c r="B18" s="32"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="40" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" s="40"/>
-      <c r="H18" s="40"/>
-      <c r="I18" s="40"/>
-      <c r="J18" s="32"/>
-      <c r="K18" s="32"/>
-      <c r="L18" s="32"/>
-      <c r="M18" s="32"/>
+      <c r="G18" s="53"/>
+      <c r="H18" s="53"/>
+      <c r="I18" s="53"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="17"/>
+      <c r="L18" s="17"/>
+      <c r="M18" s="17"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3"/>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3"/>
@@ -1263,37 +1269,37 @@
     <row r="26" spans="1:13" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A2:M3"/>
-    <mergeCell ref="A5:M5"/>
-    <mergeCell ref="C6:H6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="C7:H7"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="F8:H8"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="F11:H11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="F13:H13"/>
+    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="A16:M16"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="I10:J10"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="F9:H9"/>
     <mergeCell ref="I9:J9"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="A16:M16"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="F11:H11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="F13:H13"/>
-    <mergeCell ref="I13:J13"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="A2:M3"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="C6:H6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="C7:H7"/>
   </mergeCells>
   <pageMargins left="0.43000000000000005" right="0.4" top="0.28999999999999998" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="85" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="81" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
changes made in reports generation salary payroll
</commit_message>
<xml_diff>
--- a/public/templates/cos/payslip.xlsx
+++ b/public/templates/cos/payslip.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DOST\OneDrive\Documents\COS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DOST\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCD1AE34-D6E2-4B9E-8433-93BDDCD37645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{595A4AA0-ED57-4760-AD87-B895118EE658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4D00BDC9-532D-4D12-A161-F58336A59D96}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="PAYSLIP" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">PAYSLIP!$A$1:$M$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">PAYSLIP!$A$1:$M$17</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -84,7 +84,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-[$₱-3409]* #,##0.00_-;\-[$₱-3409]* #,##0.00_-;_-[$₱-3409]* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -158,14 +158,6 @@
     </font>
     <font>
       <sz val="8"/>
-      <color theme="1"/>
-      <name val="Courier New"/>
-      <family val="3"/>
-    </font>
-    <font>
-      <b/>
-      <u val="singleAccounting"/>
-      <sz val="10"/>
       <color theme="1"/>
       <name val="Courier New"/>
       <family val="3"/>
@@ -337,7 +329,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
@@ -359,68 +351,90 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -442,57 +456,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -593,73 +556,43 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>434340</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>99060</xdr:rowOff>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>297180</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>53340</xdr:rowOff>
+      <xdr:colOff>282081</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>38128</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 68">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9C77C983-713F-4717-AD75-6D8DE288166E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BE03C696-E80F-A14E-3450-FB5FC1EEA936}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
+      <xdr:spPr>
         <a:xfrm>
-          <a:off x="3649980" y="3017520"/>
-          <a:ext cx="1623060" cy="320040"/>
+          <a:off x="3634740" y="2247900"/>
+          <a:ext cx="1623201" cy="320068"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -979,36 +912,36 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
+      <c r="B2" s="44"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
+      <c r="F2" s="44"/>
+      <c r="G2" s="44"/>
+      <c r="H2" s="44"/>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="44"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="44"/>
     </row>
     <row r="3" spans="1:13" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="36"/>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
-      <c r="J3" s="36"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="36"/>
-      <c r="M3" s="36"/>
+      <c r="A3" s="44"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="44"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="44"/>
+      <c r="G3" s="44"/>
+      <c r="H3" s="44"/>
+      <c r="I3" s="44"/>
+      <c r="J3" s="44"/>
+      <c r="K3" s="44"/>
+      <c r="L3" s="44"/>
+      <c r="M3" s="44"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
@@ -1026,19 +959,19 @@
       <c r="M4" s="1"/>
     </row>
     <row r="5" spans="1:13" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="37"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="38"/>
-      <c r="G5" s="38"/>
-      <c r="H5" s="38"/>
-      <c r="I5" s="38"/>
-      <c r="J5" s="38"/>
-      <c r="K5" s="38"/>
-      <c r="L5" s="38"/>
-      <c r="M5" s="39"/>
+      <c r="A5" s="45"/>
+      <c r="B5" s="46"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="46"/>
+      <c r="I5" s="46"/>
+      <c r="J5" s="46"/>
+      <c r="K5" s="46"/>
+      <c r="L5" s="46"/>
+      <c r="M5" s="47"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
@@ -1047,14 +980,14 @@
       <c r="B6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="41"/>
-      <c r="J6" s="41"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="48"/>
+      <c r="H6" s="48"/>
+      <c r="I6" s="49"/>
+      <c r="J6" s="49"/>
       <c r="K6" s="4"/>
       <c r="L6" s="5"/>
       <c r="M6" s="6"/>
@@ -1066,12 +999,12 @@
       <c r="B7" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="42"/>
-      <c r="D7" s="42"/>
-      <c r="E7" s="42"/>
-      <c r="F7" s="42"/>
-      <c r="G7" s="42"/>
-      <c r="H7" s="42"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="50"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="50"/>
+      <c r="G7" s="50"/>
+      <c r="H7" s="50"/>
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
       <c r="K7" s="9"/>
@@ -1079,224 +1012,162 @@
       <c r="M7" s="10"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A8" s="43" t="s">
+      <c r="A8" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="44"/>
-      <c r="C8" s="45"/>
-      <c r="D8" s="43" t="s">
+      <c r="B8" s="42"/>
+      <c r="C8" s="43"/>
+      <c r="D8" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="45"/>
-      <c r="F8" s="43" t="s">
+      <c r="E8" s="43"/>
+      <c r="F8" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="G8" s="44"/>
-      <c r="H8" s="45"/>
-      <c r="I8" s="43" t="s">
+      <c r="G8" s="42"/>
+      <c r="H8" s="43"/>
+      <c r="I8" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="J8" s="44"/>
+      <c r="J8" s="42"/>
       <c r="K8" s="11"/>
-      <c r="L8" s="43" t="s">
+      <c r="L8" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="M8" s="45"/>
+      <c r="M8" s="43"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A9" s="49"/>
-      <c r="B9" s="50"/>
-      <c r="C9" s="50"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="50"/>
-      <c r="G9" s="50"/>
-      <c r="H9" s="50"/>
-      <c r="I9" s="50"/>
-      <c r="J9" s="50"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="22"/>
-      <c r="M9" s="19"/>
+      <c r="A9" s="37"/>
+      <c r="B9" s="38"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="39"/>
+      <c r="G9" s="39"/>
+      <c r="H9" s="39"/>
+      <c r="I9" s="40"/>
+      <c r="J9" s="40"/>
+      <c r="K9" s="20"/>
+      <c r="L9" s="20"/>
+      <c r="M9" s="18"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A10" s="46"/>
-      <c r="B10" s="47"/>
-      <c r="C10" s="47"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="48"/>
-      <c r="J10" s="48"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="18"/>
+      <c r="A10" s="34"/>
+      <c r="B10" s="35"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="35"/>
+      <c r="H10" s="35"/>
+      <c r="I10" s="36"/>
+      <c r="J10" s="36"/>
+      <c r="K10" s="21"/>
+      <c r="L10" s="17"/>
       <c r="M10" s="12"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" s="46"/>
-      <c r="B11" s="47"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="47"/>
-      <c r="G11" s="47"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="58"/>
-      <c r="J11" s="58"/>
-      <c r="K11" s="23"/>
-      <c r="L11" s="18"/>
-      <c r="M11" s="12"/>
+      <c r="A11" s="29"/>
+      <c r="B11" s="30"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="33"/>
+      <c r="J11" s="33"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="25"/>
+      <c r="M11" s="19"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="28"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="29"/>
-      <c r="E12" s="29"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="30"/>
-      <c r="K12" s="23"/>
-      <c r="L12" s="31"/>
-      <c r="M12" s="20"/>
+      <c r="A12" s="32"/>
+      <c r="B12" s="32"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="32"/>
+      <c r="K12" s="32"/>
+      <c r="L12" s="32"/>
+      <c r="M12" s="32"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" s="59"/>
-      <c r="B13" s="58"/>
-      <c r="C13" s="58"/>
-      <c r="D13" s="23"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="58"/>
-      <c r="G13" s="58"/>
-      <c r="H13" s="58"/>
-      <c r="I13" s="58"/>
-      <c r="J13" s="58"/>
-      <c r="K13" s="23"/>
-      <c r="L13" s="23"/>
-      <c r="M13" s="20"/>
-    </row>
-    <row r="14" spans="1:13" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="32"/>
-      <c r="B14" s="27"/>
-      <c r="C14" s="27"/>
-      <c r="D14" s="23"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="27"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="33"/>
-      <c r="M14" s="20"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" s="54"/>
-      <c r="B15" s="55"/>
-      <c r="C15" s="55"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="56"/>
-      <c r="G15" s="56"/>
-      <c r="H15" s="56"/>
-      <c r="I15" s="35"/>
-      <c r="J15" s="35"/>
-      <c r="K15" s="35"/>
-      <c r="L15" s="35"/>
-      <c r="M15" s="21"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" s="57"/>
-      <c r="B16" s="57"/>
-      <c r="C16" s="57"/>
-      <c r="D16" s="57"/>
-      <c r="E16" s="57"/>
-      <c r="F16" s="57"/>
-      <c r="G16" s="57"/>
-      <c r="H16" s="57"/>
-      <c r="I16" s="57"/>
-      <c r="J16" s="57"/>
-      <c r="K16" s="57"/>
-      <c r="L16" s="57"/>
-      <c r="M16" s="57"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A17" s="14"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="51" t="s">
+      <c r="A13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="D17" s="51"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="52" t="s">
+      <c r="D13" s="26"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="G17" s="52"/>
-      <c r="H17" s="52"/>
-      <c r="I17" s="52"/>
-      <c r="J17" s="16"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="14"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A18" s="17"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="53" t="s">
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="13"/>
+      <c r="L13" s="13"/>
+      <c r="M13" s="13"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A14" s="16"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="G18" s="53"/>
-      <c r="H18" s="53"/>
-      <c r="I18" s="53"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3"/>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3"/>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3"/>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3"/>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3"/>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3"/>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="16"/>
+      <c r="L14" s="16"/>
+      <c r="M14" s="16"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3"/>
+    <row r="17" x14ac:dyDescent="0.3"/>
+    <row r="18" x14ac:dyDescent="0.3"/>
+    <row r="19" x14ac:dyDescent="0.3"/>
+    <row r="20" x14ac:dyDescent="0.3"/>
+    <row r="21" x14ac:dyDescent="0.3"/>
+    <row r="22" x14ac:dyDescent="0.3"/>
+    <row r="23" x14ac:dyDescent="0.3"/>
+    <row r="24" x14ac:dyDescent="0.3"/>
+    <row r="25" x14ac:dyDescent="0.3"/>
+    <row r="26" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="28">
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="F11:H11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="F13:H13"/>
-    <mergeCell ref="I13:J13"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="A16:M16"/>
+  <mergeCells count="22">
+    <mergeCell ref="A2:M3"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="C6:H6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="C7:H7"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="L8:M8"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="I10:J10"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="F9:H9"/>
     <mergeCell ref="I9:J9"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="F8:H8"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="A2:M3"/>
-    <mergeCell ref="A5:M5"/>
-    <mergeCell ref="C6:H6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="C7:H7"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="F11:H11"/>
+    <mergeCell ref="A12:M12"/>
+    <mergeCell ref="I11:J11"/>
   </mergeCells>
   <pageMargins left="0.43000000000000005" right="0.4" top="0.28999999999999998" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="81" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fixed and redesign payslip for cos
</commit_message>
<xml_diff>
--- a/public/templates/cos/payslip.xlsx
+++ b/public/templates/cos/payslip.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DOST\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jdrinon\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EC36978-4B0D-4E6A-B9F4-6EE38DE640B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A598452-8FCE-4C3C-84A6-5AA4088E1AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4D00BDC9-532D-4D12-A161-F58336A59D96}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{4D00BDC9-532D-4D12-A161-F58336A59D96}"/>
   </bookViews>
   <sheets>
     <sheet name="PAYSLIP" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">PAYSLIP!$A$1:$M$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">PAYSLIP!$A$1:$O$20</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
   <si>
     <t xml:space="preserve">      TECHNOLOGY APPLICATION AND PROMOTION INSTITUTE</t>
   </si>
@@ -66,12 +66,6 @@
     <t>NET AMOUNT</t>
   </si>
   <si>
-    <t>Certified Correct:</t>
-  </si>
-  <si>
-    <t>AO V - HR Section</t>
-  </si>
-  <si>
     <t>REMARKS</t>
   </si>
 </sst>
@@ -80,9 +74,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="44" formatCode="_-&quot;₱&quot;* #,##0.00_-;\-&quot;₱&quot;* #,##0.00_-;_-&quot;₱&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="_-[$₱-3409]* #,##0.00_-;\-[$₱-3409]* #,##0.00_-;_-[$₱-3409]* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-&quot;₱&quot;* #,##0.00_-;\-&quot;₱&quot;* #,##0.00_-;_-&quot;₱&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-[$₱-3409]* #,##0.00_-;\-[$₱-3409]* #,##0.00_-;_-[$₱-3409]* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -327,7 +321,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -357,7 +351,7 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -372,10 +366,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -388,9 +382,33 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -415,7 +433,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -424,7 +442,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -436,32 +454,8 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -494,9 +488,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>144435</xdr:colOff>
+      <xdr:colOff>136815</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>220980</xdr:rowOff>
+      <xdr:rowOff>207645</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -852,60 +846,60 @@
   <sheetPr codeName="Sheet37">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
-  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.4" zeroHeight="1" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:P17"/>
+  <sheetFormatPr defaultColWidth="0" defaultRowHeight="14.5" zeroHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.5546875" customWidth="1"/>
+    <col min="1" max="1" width="17.54296875" customWidth="1"/>
     <col min="2" max="2" width="2" customWidth="1"/>
-    <col min="3" max="3" width="9.109375" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" customWidth="1"/>
-    <col min="5" max="5" width="2.33203125" customWidth="1"/>
-    <col min="6" max="7" width="9.109375" customWidth="1"/>
-    <col min="8" max="8" width="7.44140625" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" customWidth="1"/>
-    <col min="10" max="10" width="7.109375" customWidth="1"/>
-    <col min="11" max="11" width="2.33203125" customWidth="1"/>
-    <col min="12" max="12" width="16.6640625" customWidth="1"/>
-    <col min="13" max="13" width="8.21875" customWidth="1"/>
-    <col min="14" max="15" width="9.109375" customWidth="1"/>
+    <col min="3" max="3" width="9.08984375" customWidth="1"/>
+    <col min="4" max="4" width="15.90625" customWidth="1"/>
+    <col min="5" max="5" width="2.36328125" customWidth="1"/>
+    <col min="6" max="7" width="9.08984375" customWidth="1"/>
+    <col min="8" max="8" width="7.453125" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" customWidth="1"/>
+    <col min="10" max="10" width="7.08984375" customWidth="1"/>
+    <col min="11" max="11" width="2.36328125" customWidth="1"/>
+    <col min="12" max="12" width="16.6328125" customWidth="1"/>
+    <col min="13" max="13" width="8.1796875" customWidth="1"/>
+    <col min="14" max="15" width="9.08984375" customWidth="1"/>
     <col min="16" max="16" width="0" hidden="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.109375" hidden="1"/>
+    <col min="17" max="16384" width="9.08984375" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A2" s="46" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A2" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-    </row>
-    <row r="3" spans="1:15" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="46"/>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
-      <c r="K3" s="46"/>
-      <c r="L3" s="46"/>
-      <c r="M3" s="46"/>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+    </row>
+    <row r="3" spans="1:15" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="30"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
+      <c r="K3" s="30"/>
+      <c r="L3" s="30"/>
+      <c r="M3" s="30"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -920,225 +914,204 @@
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
     </row>
-    <row r="5" spans="1:15" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="47"/>
-      <c r="B5" s="48"/>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="48"/>
-      <c r="F5" s="48"/>
-      <c r="G5" s="48"/>
-      <c r="H5" s="48"/>
-      <c r="I5" s="48"/>
-      <c r="J5" s="48"/>
-      <c r="K5" s="48"/>
-      <c r="L5" s="48"/>
-      <c r="M5" s="49"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="33" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="31"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="32"/>
+      <c r="M5" s="33"/>
+    </row>
+    <row r="6" spans="1:15" ht="15" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="50"/>
-      <c r="D6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="50"/>
-      <c r="I6" s="51"/>
-      <c r="J6" s="51"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="35"/>
+      <c r="J6" s="35"/>
       <c r="K6" s="4"/>
       <c r="L6" s="5"/>
       <c r="M6" s="6"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="15" x14ac:dyDescent="0.4">
       <c r="A7" s="7" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="52"/>
-      <c r="D7" s="52"/>
-      <c r="E7" s="52"/>
-      <c r="F7" s="52"/>
-      <c r="G7" s="52"/>
-      <c r="H7" s="52"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
       <c r="K7" s="9"/>
       <c r="L7" s="9"/>
       <c r="M7" s="10"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="15" x14ac:dyDescent="0.4">
       <c r="A8" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="45"/>
-      <c r="C8" s="28"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="29"/>
       <c r="D8" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="28"/>
+      <c r="E8" s="29"/>
       <c r="F8" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="G8" s="45"/>
-      <c r="H8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="29"/>
       <c r="I8" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="J8" s="45"/>
+      <c r="J8" s="28"/>
       <c r="K8" s="11"/>
       <c r="L8" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="M8" s="28"/>
+      <c r="M8" s="29"/>
       <c r="N8" s="27" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
-      <c r="O8" s="28"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A9" s="41"/>
-      <c r="B9" s="42"/>
-      <c r="C9" s="42"/>
+      <c r="O8" s="29"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A9" s="49"/>
+      <c r="B9" s="50"/>
+      <c r="C9" s="50"/>
       <c r="D9" s="21"/>
       <c r="E9" s="21"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="43"/>
-      <c r="H9" s="43"/>
-      <c r="I9" s="44"/>
-      <c r="J9" s="44"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="51"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="52"/>
+      <c r="J9" s="52"/>
       <c r="K9" s="20"/>
       <c r="L9" s="20"/>
       <c r="M9" s="18"/>
-      <c r="N9" s="29"/>
-      <c r="O9" s="29"/>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A10" s="38"/>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
+      <c r="N9" s="37"/>
+      <c r="O9" s="37"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A10" s="46"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
       <c r="D10" s="22"/>
       <c r="E10" s="23"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="40"/>
-      <c r="J10" s="40"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="48"/>
+      <c r="J10" s="48"/>
       <c r="K10" s="21"/>
       <c r="L10" s="17"/>
       <c r="M10" s="12"/>
-      <c r="N10" s="30"/>
-      <c r="O10" s="30"/>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A11" s="33"/>
-      <c r="B11" s="34"/>
-      <c r="C11" s="34"/>
+      <c r="N10" s="38"/>
+      <c r="O10" s="38"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A11" s="41"/>
+      <c r="B11" s="42"/>
+      <c r="C11" s="42"/>
       <c r="D11" s="24"/>
       <c r="E11" s="24"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="37"/>
-      <c r="J11" s="37"/>
+      <c r="F11" s="43"/>
+      <c r="G11" s="43"/>
+      <c r="H11" s="43"/>
+      <c r="I11" s="45"/>
+      <c r="J11" s="45"/>
       <c r="K11" s="25"/>
       <c r="L11" s="25"/>
       <c r="M11" s="19"/>
-      <c r="N11" s="30"/>
-      <c r="O11" s="30"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A12" s="36"/>
-      <c r="B12" s="36"/>
-      <c r="C12" s="36"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="36"/>
-      <c r="F12" s="36"/>
-      <c r="G12" s="36"/>
-      <c r="H12" s="36"/>
-      <c r="I12" s="36"/>
-      <c r="J12" s="36"/>
-      <c r="K12" s="36"/>
-      <c r="L12" s="36"/>
-      <c r="M12" s="36"/>
-      <c r="N12" s="30"/>
-      <c r="O12" s="30"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N11" s="38"/>
+      <c r="O11" s="38"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="A12" s="44"/>
+      <c r="B12" s="44"/>
+      <c r="C12" s="44"/>
+      <c r="D12" s="44"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="44"/>
+      <c r="G12" s="44"/>
+      <c r="H12" s="44"/>
+      <c r="I12" s="44"/>
+      <c r="J12" s="44"/>
+      <c r="K12" s="44"/>
+      <c r="L12" s="44"/>
+      <c r="M12" s="44"/>
+      <c r="N12" s="38"/>
+      <c r="O12" s="38"/>
+    </row>
+    <row r="13" spans="1:15" ht="15" x14ac:dyDescent="0.4">
       <c r="A13" s="13"/>
       <c r="B13" s="13"/>
-      <c r="C13" s="26" t="s">
-        <v>9</v>
-      </c>
+      <c r="C13" s="26"/>
       <c r="D13" s="26"/>
       <c r="E13" s="14"/>
-      <c r="F13" s="31"/>
-      <c r="G13" s="31"/>
-      <c r="H13" s="31"/>
-      <c r="I13" s="31"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="39"/>
+      <c r="H13" s="39"/>
+      <c r="I13" s="39"/>
       <c r="J13" s="15"/>
       <c r="K13" s="13"/>
       <c r="L13" s="13"/>
       <c r="M13" s="13"/>
-      <c r="N13" s="30"/>
-      <c r="O13" s="30"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="N13" s="38"/>
+      <c r="O13" s="38"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" s="16"/>
       <c r="B14" s="16"/>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
-      <c r="F14" s="32" t="s">
-        <v>10</v>
-      </c>
-      <c r="G14" s="32"/>
-      <c r="H14" s="32"/>
-      <c r="I14" s="32"/>
+      <c r="F14" s="40"/>
+      <c r="G14" s="40"/>
+      <c r="H14" s="40"/>
+      <c r="I14" s="40"/>
       <c r="J14" s="16"/>
       <c r="K14" s="16"/>
       <c r="L14" s="16"/>
       <c r="M14" s="16"/>
-      <c r="N14" s="30"/>
-      <c r="O14" s="30"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="N15" s="30"/>
-      <c r="O15" s="30"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="N16" s="30"/>
-      <c r="O16" s="30"/>
-    </row>
-    <row r="17" spans="14:15" x14ac:dyDescent="0.3">
-      <c r="N17" s="30"/>
-      <c r="O17" s="30"/>
-    </row>
-    <row r="18" spans="14:15" x14ac:dyDescent="0.3"/>
-    <row r="19" spans="14:15" x14ac:dyDescent="0.3"/>
-    <row r="20" spans="14:15" x14ac:dyDescent="0.3"/>
-    <row r="21" spans="14:15" x14ac:dyDescent="0.3"/>
-    <row r="22" spans="14:15" x14ac:dyDescent="0.3"/>
-    <row r="23" spans="14:15" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="14:15" x14ac:dyDescent="0.3"/>
-    <row r="25" spans="14:15" x14ac:dyDescent="0.3"/>
-    <row r="26" spans="14:15" x14ac:dyDescent="0.3"/>
+      <c r="N14" s="38"/>
+      <c r="O14" s="38"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="N15" s="38"/>
+      <c r="O15" s="38"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="N16" s="38"/>
+      <c r="O16" s="38"/>
+    </row>
+    <row r="17" spans="14:15" x14ac:dyDescent="0.35">
+      <c r="N17" s="38"/>
+      <c r="O17" s="38"/>
+    </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="F8:H8"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="A2:M3"/>
-    <mergeCell ref="A5:M5"/>
-    <mergeCell ref="C6:H6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="C7:H7"/>
     <mergeCell ref="N8:O8"/>
     <mergeCell ref="N9:O17"/>
     <mergeCell ref="F13:I13"/>
@@ -1155,9 +1128,17 @@
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="D8:E8"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="A2:M3"/>
+    <mergeCell ref="A5:M5"/>
+    <mergeCell ref="C6:H6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="C7:H7"/>
   </mergeCells>
   <pageMargins left="0.43000000000000005" right="0.4" top="0.28999999999999998" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="82" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="72" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>